<commit_message>
Agrega descripcion de bianchi
</commit_message>
<xml_diff>
--- a/Resultados_correcciones/Entregable/Reporte_Dip_SinInc_vf_2.xlsx
+++ b/Resultados_correcciones/Entregable/Reporte_Dip_SinInc_vf_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/be16ff5b34c21876/Documents/Trabajo/EstrategiaSur/Proyeccion-electoral-congreso/Resultados_correcciones/Entregable/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="202" documentId="13_ncr:1_{96D5EEAF-DB2C-4CCB-9C95-40C8884B4BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0BE3E3BE-3209-4D91-8423-AF3FA6635AB8}"/>
+  <xr:revisionPtr revIDLastSave="203" documentId="13_ncr:1_{96D5EEAF-DB2C-4CCB-9C95-40C8884B4BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66C309EF-3098-4E52-9A8F-C638449B2C2D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="16" xr2:uid="{85AAF8D7-1A96-46DE-A921-B4694576F524}"/>
   </bookViews>
@@ -256,45 +256,6 @@
   </si>
   <si>
     <t>AMA</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Algunos puntos a tener en cuenta sobre los resultados del modelo:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
--  Los resultados presentados son el producto de un modelo mixto que combina variables determinísticas y probabilísticas. Las variables determinísticas están basadas en datos observables y predecibles, mientras que las probabilísticas buscan capturar aquellas dinámicas que no se pueden predecir completamente a partir de mediciones conocidas. Esto permite modelar incertidumbres inherentes al sistema. Aunque los resultados no representan la realidad al 100%, se estima que los resultados reales estarán dentro de un rango cercano, considerando un margen de error razonable.
-- Carlos Bianchi se considera como Independiente y Christian Matheson como Evopoli
-- Hay que estar atentos a la definición que tome Bianchi. El modelo no fue capaz de predecir la votación de su figura
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>- Para observar el modelo con el factor de incumbencias revisar el archivo "Reporte_Dip.xlsx"</t>
-    </r>
   </si>
   <si>
     <r>
@@ -747,6 +708,45 @@
   <si>
     <t>POP</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Algunos puntos a tener en cuenta sobre los resultados del modelo:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+-  Los resultados presentados son el producto de un modelo mixto que combina variables determinísticas y probabilísticas. Las variables determinísticas están basadas en datos observables y predecibles, mientras que las probabilísticas buscan capturar aquellas dinámicas que no se pueden predecir completamente a partir de mediciones conocidas. Esto permite modelar incertidumbres inherentes al sistema. Aunque los resultados no representan la realidad al 100%, se estima que los resultados reales estarán dentro de un rango cercano, considerando un margen de error razonable.
+- Carlos Bianchi se considera como Independiente y Christian Matheson como Evopoli
+-Modelo ajustado que incorpora efecto caudillo de Bianchi
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>- Para observar el modelo con el factor de incumbencias revisar el archivo "Reporte_Dip.xlsx"</t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -1184,6 +1184,27 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
@@ -1191,7 +1212,157 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1212,7 +1383,42 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1226,14 +1432,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
+          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1241,13 +1440,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1306,7 +1498,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1320,7 +1512,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1328,13 +1527,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1363,6 +1555,243 @@
       <fill>
         <patternFill>
           <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1432,6 +1861,149 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFABAB"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
@@ -1440,13 +2012,6 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1470,7 +2035,28 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1484,593 +2070,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFABAB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFABAB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFABAB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFABAB"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF0070C0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00B050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2112,7 +2112,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FF7030A0"/>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2126,28 +2140,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="5" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2175,6 +2168,13 @@
     <dxf>
       <fill>
         <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
           <bgColor theme="5" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
@@ -2182,14 +2182,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="2" tint="-0.24994659260841701"/>
+          <bgColor rgb="FFFFC000"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC000"/>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -27314,13 +27314,13 @@
         <v>36</v>
       </c>
       <c r="AD3" s="31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AE3" s="31" t="s">
         <v>36</v>
       </c>
       <c r="AH3" s="31" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="AI3" s="31" t="s">
         <v>36</v>
@@ -28684,43 +28684,43 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B4:C27">
-    <cfRule type="cellIs" dxfId="141" priority="136" operator="equal">
+    <cfRule type="cellIs" dxfId="141" priority="142" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="140" priority="136" operator="equal">
       <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="140" priority="137" operator="equal">
-      <formula>"p6"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="139" priority="138" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="138" priority="139" operator="equal">
+    <cfRule type="cellIs" dxfId="138" priority="137" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="137" priority="139" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="137" priority="140" operator="equal">
+    <cfRule type="cellIs" dxfId="136" priority="140" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="136" priority="141" operator="equal">
+    <cfRule type="cellIs" dxfId="135" priority="141" operator="equal">
       <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="135" priority="142" operator="equal">
-      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:G27">
-    <cfRule type="cellIs" dxfId="134" priority="94" operator="equal">
-      <formula>"p7"</formula>
+    <cfRule type="cellIs" dxfId="134" priority="98" operator="equal">
+      <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="133" priority="95" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="133" priority="97" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="132" priority="96" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="131" priority="97" operator="equal">
-      <formula>"p4"</formula>
+    <cfRule type="cellIs" dxfId="131" priority="95" operator="equal">
+      <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="130" priority="98" operator="equal">
-      <formula>"p3"</formula>
+    <cfRule type="cellIs" dxfId="130" priority="94" operator="equal">
+      <formula>"p7"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="129" priority="99" operator="equal">
       <formula>"p2"</formula>
@@ -28741,31 +28741,31 @@
     <cfRule type="cellIs" dxfId="125" priority="130" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="124" priority="131" operator="equal">
-      <formula>"p5"</formula>
+    <cfRule type="cellIs" dxfId="124" priority="135" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="123" priority="132" operator="equal">
-      <formula>"p4"</formula>
+    <cfRule type="cellIs" dxfId="123" priority="134" operator="equal">
+      <formula>"p2"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="122" priority="133" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="121" priority="134" operator="equal">
-      <formula>"p2"</formula>
+    <cfRule type="cellIs" dxfId="121" priority="132" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="120" priority="135" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="120" priority="131" operator="equal">
+      <formula>"p5"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:K27 AD5:AE27">
-    <cfRule type="cellIs" dxfId="119" priority="80" operator="equal">
+    <cfRule type="cellIs" dxfId="119" priority="82" operator="equal">
+      <formula>"p11"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="118" priority="80" operator="equal">
       <formula>"p13"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="118" priority="81" operator="equal">
+    <cfRule type="cellIs" dxfId="117" priority="81" operator="equal">
       <formula>"p12"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="117" priority="82" operator="equal">
-      <formula>"p11"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="116" priority="83" operator="equal">
       <formula>"p10"</formula>
@@ -28775,69 +28775,69 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K27 AE5:AE27">
-    <cfRule type="cellIs" dxfId="114" priority="85" operator="equal">
-      <formula>"p8"</formula>
+    <cfRule type="cellIs" dxfId="114" priority="92" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="113" priority="86" operator="equal">
+    <cfRule type="cellIs" dxfId="113" priority="89" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="112" priority="91" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="111" priority="90" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="110" priority="88" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="109" priority="87" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="108" priority="86" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="112" priority="87" operator="equal">
-      <formula>"p6"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="111" priority="88" operator="equal">
-      <formula>"p5"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="110" priority="89" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="109" priority="90" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="108" priority="91" operator="equal">
-      <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="107" priority="92" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="107" priority="85" operator="equal">
+      <formula>"p8"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N4:O4">
-    <cfRule type="cellIs" dxfId="106" priority="122" operator="equal">
+    <cfRule type="cellIs" dxfId="106" priority="125" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="105" priority="128" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="104" priority="127" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="103" priority="126" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="102" priority="123" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="101" priority="122" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="105" priority="123" operator="equal">
-      <formula>"p6"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="104" priority="124" operator="equal">
+    <cfRule type="cellIs" dxfId="100" priority="124" operator="equal">
       <formula>"p5"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="103" priority="125" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="102" priority="126" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="101" priority="127" operator="equal">
-      <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="100" priority="128" operator="equal">
-      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:O27">
-    <cfRule type="cellIs" dxfId="99" priority="67" operator="equal">
+    <cfRule type="cellIs" dxfId="99" priority="71" operator="equal">
+      <formula>"p9"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="98" priority="69" operator="equal">
+      <formula>"p11"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="97" priority="68" operator="equal">
+      <formula>"p12"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="96" priority="67" operator="equal">
       <formula>"p13"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="98" priority="68" operator="equal">
-      <formula>"p12"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="97" priority="69" operator="equal">
-      <formula>"p11"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="96" priority="70" operator="equal">
+    <cfRule type="cellIs" dxfId="95" priority="70" operator="equal">
       <formula>"p10"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="95" priority="71" operator="equal">
-      <formula>"p9"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O27">
@@ -28870,106 +28870,106 @@
     <cfRule type="cellIs" dxfId="86" priority="115" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="85" priority="116" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="85" priority="121" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="117" operator="equal">
+    <cfRule type="cellIs" dxfId="84" priority="120" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="83" priority="119" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="82" priority="118" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="81" priority="117" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="83" priority="118" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="82" priority="119" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="81" priority="120" operator="equal">
-      <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="80" priority="121" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="80" priority="116" operator="equal">
+      <formula>"p6"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R5:S27">
-    <cfRule type="cellIs" dxfId="79" priority="54" operator="equal">
-      <formula>"p13"</formula>
+    <cfRule type="cellIs" dxfId="79" priority="58" operator="equal">
+      <formula>"p9"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="78" priority="55" operator="equal">
       <formula>"p12"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="77" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="77" priority="57" operator="equal">
+      <formula>"p10"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="76" priority="56" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="57" operator="equal">
-      <formula>"p10"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="75" priority="58" operator="equal">
-      <formula>"p9"</formula>
+    <cfRule type="cellIs" dxfId="75" priority="54" operator="equal">
+      <formula>"p13"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S5:S27">
-    <cfRule type="cellIs" dxfId="74" priority="59" operator="equal">
-      <formula>"p8"</formula>
+    <cfRule type="cellIs" dxfId="74" priority="63" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="73" priority="60" operator="equal">
-      <formula>"p7"</formula>
+    <cfRule type="cellIs" dxfId="73" priority="62" operator="equal">
+      <formula>"p5"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="72" priority="61" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="71" priority="62" operator="equal">
-      <formula>"p5"</formula>
+    <cfRule type="cellIs" dxfId="71" priority="60" operator="equal">
+      <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="63" operator="equal">
-      <formula>"p4"</formula>
+    <cfRule type="cellIs" dxfId="70" priority="59" operator="equal">
+      <formula>"p8"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="69" priority="64" operator="equal">
-      <formula>"p3"</formula>
+    <cfRule type="cellIs" dxfId="69" priority="66" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="68" priority="65" operator="equal">
       <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="67" priority="66" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="67" priority="64" operator="equal">
+      <formula>"p3"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V4:W4">
-    <cfRule type="cellIs" dxfId="66" priority="108" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="65" priority="109" operator="equal">
+    <cfRule type="cellIs" dxfId="66" priority="109" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="110" operator="equal">
+    <cfRule type="cellIs" dxfId="65" priority="114" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="64" priority="113" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="63" priority="112" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="62" priority="111" operator="equal">
+      <formula>"p4"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="61" priority="110" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="63" priority="111" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="112" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="61" priority="113" operator="equal">
-      <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="114" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="60" priority="108" operator="equal">
+      <formula>"p7"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V5:W27">
     <cfRule type="cellIs" dxfId="59" priority="41" operator="equal">
       <formula>"p13"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="42" operator="equal">
-      <formula>"p12"</formula>
+    <cfRule type="cellIs" dxfId="58" priority="44" operator="equal">
+      <formula>"p10"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="57" priority="43" operator="equal">
+    <cfRule type="cellIs" dxfId="57" priority="45" operator="equal">
+      <formula>"p9"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="56" priority="43" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="44" operator="equal">
-      <formula>"p10"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="45" operator="equal">
-      <formula>"p9"</formula>
+    <cfRule type="cellIs" dxfId="55" priority="42" operator="equal">
+      <formula>"p12"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W5:W27">
@@ -28991,22 +28991,22 @@
     <cfRule type="cellIs" dxfId="49" priority="51" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="52" operator="equal">
+    <cfRule type="cellIs" dxfId="48" priority="53" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="47" priority="52" operator="equal">
       <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="47" priority="53" operator="equal">
-      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z4:AA4">
-    <cfRule type="cellIs" dxfId="46" priority="101" operator="equal">
-      <formula>"p7"</formula>
+    <cfRule type="cellIs" dxfId="46" priority="103" operator="equal">
+      <formula>"p5"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="45" priority="102" operator="equal">
       <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="103" operator="equal">
-      <formula>"p5"</formula>
+    <cfRule type="cellIs" dxfId="44" priority="101" operator="equal">
+      <formula>"p7"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="43" priority="104" operator="equal">
       <formula>"p4"</formula>
@@ -29031,126 +29031,126 @@
     <cfRule type="cellIs" dxfId="37" priority="30" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="32" operator="equal">
+      <formula>"p9"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="35" priority="31" operator="equal">
       <formula>"p10"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="35" priority="32" operator="equal">
-      <formula>"p9"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA5:AA27">
-    <cfRule type="cellIs" dxfId="34" priority="33" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="35" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="40" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="39" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="31" priority="38" operator="equal">
+      <formula>"p3"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="36" operator="equal">
+      <formula>"p5"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="34" operator="equal">
+      <formula>"p7"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="33" operator="equal">
       <formula>"p8"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="33" priority="34" operator="equal">
-      <formula>"p7"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="35" operator="equal">
-      <formula>"p6"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="36" operator="equal">
-      <formula>"p5"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="37" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="37" operator="equal">
       <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="29" priority="38" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="39" operator="equal">
-      <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="40" operator="equal">
-      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD4:AE4">
-    <cfRule type="cellIs" dxfId="26" priority="21" operator="equal">
-      <formula>"p7"</formula>
+    <cfRule type="cellIs" dxfId="26" priority="25" operator="equal">
+      <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="22" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="25" priority="24" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="24" priority="23" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="24" operator="equal">
-      <formula>"p4"</formula>
+    <cfRule type="cellIs" dxfId="23" priority="22" operator="equal">
+      <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="25" operator="equal">
-      <formula>"p3"</formula>
+    <cfRule type="cellIs" dxfId="22" priority="21" operator="equal">
+      <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="26" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="27" operator="equal">
+      <formula>"p1"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="26" operator="equal">
       <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="27" operator="equal">
-      <formula>"p1"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH4:AI4">
-    <cfRule type="cellIs" dxfId="19" priority="14" operator="equal">
-      <formula>"p7"</formula>
+    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
+      <formula>"p2"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="15" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="18" priority="17" operator="equal">
+      <formula>"p4"</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="17" priority="16" operator="equal">
       <formula>"p5"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="17" operator="equal">
-      <formula>"p4"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="18" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="18" operator="equal">
       <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="19" operator="equal">
-      <formula>"p2"</formula>
+    <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
+      <formula>"p6"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="20" operator="equal">
       <formula>"p1"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="equal">
+      <formula>"p7"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH5:AI27">
-    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
-      <formula>"p13"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
       <formula>"p12"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="3" operator="equal">
       <formula>"p11"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="4" operator="equal">
       <formula>"p10"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
       <formula>"p9"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+      <formula>"p13"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI5:AI27">
     <cfRule type="cellIs" dxfId="7" priority="6" operator="equal">
       <formula>"p8"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
+      <formula>"p6"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>"p7"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="8" operator="equal">
-      <formula>"p6"</formula>
+    <cfRule type="cellIs" dxfId="4" priority="11" operator="equal">
+      <formula>"p3"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="9" operator="equal">
-      <formula>"p5"</formula>
+    <cfRule type="cellIs" dxfId="3" priority="13" operator="equal">
+      <formula>"p1"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="12" operator="equal">
+      <formula>"p2"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="10" operator="equal">
       <formula>"p4"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="11" operator="equal">
-      <formula>"p3"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="12" operator="equal">
-      <formula>"p2"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="13" operator="equal">
-      <formula>"p1"</formula>
+    <cfRule type="cellIs" dxfId="0" priority="9" operator="equal">
+      <formula>"p5"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -29467,7 +29467,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -29493,7 +29493,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -29520,7 +29520,7 @@
     <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:9" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -29973,7 +29973,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -30002,7 +30002,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -30032,7 +30032,7 @@
     <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -30458,7 +30458,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>0</v>
@@ -30484,7 +30484,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>0</v>
@@ -30511,7 +30511,7 @@
     <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:9" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -30995,7 +30995,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>0</v>
@@ -31027,7 +31027,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>0</v>
@@ -31060,7 +31060,7 @@
     <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -31563,7 +31563,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -31595,7 +31595,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -31628,7 +31628,7 @@
     <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -32064,7 +32064,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -32090,7 +32090,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -32117,7 +32117,7 @@
     <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:9" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -32532,7 +32532,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -32558,7 +32558,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -32585,7 +32585,7 @@
     <row r="15" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:9" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -33100,7 +33100,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <f>VLOOKUP($A$1,[9]resultados_integracion_partido_!$A$1:$Z$29,MATCH(C$2,[9]resultados_integracion_partido_!$A$1:$Z$1,0),FALSE)</f>
@@ -33137,7 +33137,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <f>VLOOKUP($A$1,[10]resultados_integracion_partido_!$A$1:$Z$29,MATCH(C$2,[10]resultados_integracion_partido_!$A$1:$Z$1,0),FALSE)</f>
@@ -33175,7 +33175,7 @@
     <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -33330,7 +33330,7 @@
         <v>12</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>25</v>
@@ -33354,7 +33354,7 @@
         <v>16</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>14</v>
@@ -34003,7 +34003,7 @@
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B12" s="1">
         <v>0</v>
@@ -34077,7 +34077,7 @@
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B13" s="1">
         <v>0</v>
@@ -34628,7 +34628,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>0</v>
@@ -34669,7 +34669,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>0</v>
@@ -34711,7 +34711,7 @@
     <row r="15" spans="1:14" ht="6.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:14" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -35244,7 +35244,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -35276,7 +35276,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -35309,7 +35309,7 @@
     <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -35849,7 +35849,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -35884,7 +35884,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -35920,7 +35920,7 @@
     <row r="15" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:12" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -36435,7 +36435,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>2</v>
@@ -36467,7 +36467,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>2</v>
@@ -36500,7 +36500,7 @@
     <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -36972,7 +36972,7 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>3</v>
@@ -37001,7 +37001,7 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>3</v>
@@ -37031,7 +37031,7 @@
     <row r="15" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:10" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -37525,7 +37525,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -37557,7 +37557,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -37590,7 +37590,7 @@
     <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>
@@ -38095,7 +38095,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C13" s="6">
         <v>2</v>
@@ -38127,7 +38127,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C14" s="6">
         <v>2</v>
@@ -38160,7 +38160,7 @@
     <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="16" spans="1:11" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C16" s="37"/>
       <c r="D16" s="37"/>

</xml_diff>